<commit_message>
Upgrade lightning and drum prospects with verified local firms
Replace weaker or out-of-area lightning and drum rows with locally documented companies, named principals, and published phones. Drop SEO-mill electricians, India-branded tank depots, and unverified IBC marketing sites.

Co-authored-by: anthonyleedu <anthonyleedu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Builder + Caller Masterlist - SBC 2026.xlsx
+++ b/Builder + Caller Masterlist - SBC 2026.xlsx
@@ -5068,7 +5068,7 @@
     <row r="67" ht="48" customHeight="1" s="47">
       <c r="A67" s="49" t="inlineStr">
         <is>
-          <t>Beach Electrical</t>
+          <t>Beach Electrical LLC (dba Beach Electric)</t>
         </is>
       </c>
       <c r="B67" s="49" t="inlineStr">
@@ -5078,47 +5078,47 @@
       </c>
       <c r="C67" s="49" t="inlineStr">
         <is>
-          <t>Felton, CA (Santa Cruz; serves South Bay)</t>
+          <t>Felton, CA (Santa Cruz; advertises San Jose / Bay Area work)</t>
         </is>
       </c>
       <c r="D67" s="49" t="inlineStr">
         <is>
+          <t>Jason Beach (Jason Lee Beach)</t>
+        </is>
+      </c>
+      <c r="E67" s="50" t="inlineStr">
+        <is>
+          <t>(831) 246-4014</t>
+        </is>
+      </c>
+      <c r="F67" s="49" t="inlineStr">
+        <is>
+          <t>Owner Direct</t>
+        </is>
+      </c>
+      <c r="G67" s="49" t="n">
+        <v>4</v>
+      </c>
+      <c r="H67" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E67" s="50" t="inlineStr">
-        <is>
-          <t>(831) 246-4014</t>
-        </is>
-      </c>
-      <c r="F67" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G67" s="49" t="n">
-        <v>30</v>
-      </c>
-      <c r="H67" s="49" t="inlineStr">
+      <c r="I67" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J67" s="49" t="inlineStr">
+        <is>
+          <t>https://beachelectricalca.com/services/lightning-protection-system/</t>
+        </is>
+      </c>
+      <c r="K67" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="I67" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J67" s="49" t="inlineStr">
-        <is>
-          <t>https://beachelectricalca.com/services/lightning-protection-system/</t>
-        </is>
-      </c>
-      <c r="K67" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L67" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="M67" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. C-10 electricians advertising NFPA 780 lightning-protection system design/install (air terminals, conductors, ground rods). Santa Cruz County — confirm Bay Area job mix.</t>
+          <t>Owner-direct contact is published for Jason Beach; confirm they are still the current equity owner. Closest local NFPA 780 lightning-protection installer (air terminals, conductors, ground rods, panel SPD). CSLB C-10 #1108407. LLC formed 2022; owner cites 30+ years electrical experience. Alt (408) 310-9447.</t>
         </is>
       </c>
       <c r="N67" s="49" t="inlineStr">
@@ -5143,7 +5143,7 @@
     <row r="68" ht="48" customHeight="1" s="47">
       <c r="A68" s="49" t="inlineStr">
         <is>
-          <t>Skyline Electric LLC</t>
+          <t>Bravo Communications, Inc.</t>
         </is>
       </c>
       <c r="B68" s="49" t="inlineStr">
@@ -5153,47 +5153,47 @@
       </c>
       <c r="C68" s="49" t="inlineStr">
         <is>
-          <t>Hayward, CA (Alameda)</t>
+          <t>San Jose, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D68" s="49" t="inlineStr">
         <is>
+          <t>Dennis L. Mozingo</t>
+        </is>
+      </c>
+      <c r="E68" s="50" t="inlineStr">
+        <is>
+          <t>(408) 297-8700</t>
+        </is>
+      </c>
+      <c r="F68" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G68" s="49" t="n">
+        <v>41</v>
+      </c>
+      <c r="H68" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E68" s="50" t="inlineStr">
-        <is>
-          <t>(510) 470-0520</t>
-        </is>
-      </c>
-      <c r="F68" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G68" s="49" t="n">
-        <v>10</v>
-      </c>
-      <c r="H68" s="49" t="inlineStr">
+      <c r="I68" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J68" s="49" t="inlineStr">
+        <is>
+          <t>http://www.bravobravo.com</t>
+        </is>
+      </c>
+      <c r="K68" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="I68" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J68" s="49" t="inlineStr">
-        <is>
-          <t>https://www.skylineelectricusa.com/whole-house-surge-protection</t>
-        </is>
-      </c>
-      <c r="K68" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L68" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="M68" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Advertises whole-house surge protection, panel SPD integration, and grounding/bonding. CSLB C-10 #1121036; alt (510) 512-5362. 22263 Prospect St.</t>
+          <t>Business line: ask for Dennis L. Mozingo and confirm current ownership. San Jose manufacturer/supplier of lightning and surge-protection products (Sure/Fire) plus consulting. Founded 1985. Product/consulting fit, not a typical field LPS installer. Alt (408) 270-1547.</t>
         </is>
       </c>
       <c r="N68" s="49" t="inlineStr">
@@ -5218,7 +5218,7 @@
     <row r="69" ht="48" customHeight="1" s="47">
       <c r="A69" s="49" t="inlineStr">
         <is>
-          <t>Frayer Electric Inc.</t>
+          <t>Yotta Electrical Services, Inc.</t>
         </is>
       </c>
       <c r="B69" s="49" t="inlineStr">
@@ -5228,34 +5228,32 @@
       </c>
       <c r="C69" s="49" t="inlineStr">
         <is>
-          <t>East Bay / Patterson service area, CA</t>
+          <t>San Jose, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D69" s="49" t="inlineStr">
         <is>
+          <t>Thomas Burg (CEO); Leon Badarie also listed as co-founder in some profiles</t>
+        </is>
+      </c>
+      <c r="E69" s="50" t="inlineStr">
+        <is>
+          <t>(408) 256-7653</t>
+        </is>
+      </c>
+      <c r="F69" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G69" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="H69" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E69" s="50" t="inlineStr">
-        <is>
-          <t>(510) 861-6247</t>
-        </is>
-      </c>
-      <c r="F69" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G69" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H69" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I69" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5263,12 +5261,12 @@
       </c>
       <c r="J69" s="49" t="inlineStr">
         <is>
-          <t>https://frayerelectricinc.com/services/whole-house-surge-protection/</t>
+          <t>https://yottaelectric.com/</t>
         </is>
       </c>
       <c r="K69" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@yottaelectric.com</t>
         </is>
       </c>
       <c r="L69" s="49" t="inlineStr">
@@ -5278,7 +5276,7 @@
       </c>
       <c r="M69" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. C-10 #1101008; locally owned; advertises whole-house SPD install and grounding. Confirm primary operating city and commercial mix.</t>
+          <t>Business line: ask for Thomas Burg and confirm current ownership. Dedicated commercial surge-protection and grounding-system design/install page. Started Dec 2018. SCVNECA also lists Tom Burg (408) 205-6478 / tom@yottaelectric.com.</t>
         </is>
       </c>
       <c r="N69" s="49" t="inlineStr">
@@ -5295,7 +5293,7 @@
     <row r="70" ht="48" customHeight="1" s="47">
       <c r="A70" s="49" t="inlineStr">
         <is>
-          <t>Eleos Electric</t>
+          <t>Towery Electric, Inc.</t>
         </is>
       </c>
       <c r="B70" s="49" t="inlineStr">
@@ -5305,49 +5303,47 @@
       </c>
       <c r="C70" s="49" t="inlineStr">
         <is>
-          <t>Windsor / Santa Rosa, CA (Sonoma)</t>
+          <t>Novato, CA (Marin)</t>
         </is>
       </c>
       <c r="D70" s="49" t="inlineStr">
         <is>
+          <t>Alex Towery</t>
+        </is>
+      </c>
+      <c r="E70" s="50" t="inlineStr">
+        <is>
+          <t>(415) 419-5960</t>
+        </is>
+      </c>
+      <c r="F70" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G70" s="49" t="n">
+        <v>12</v>
+      </c>
+      <c r="H70" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E70" s="50" t="inlineStr">
-        <is>
-          <t>(707) 837-6722</t>
-        </is>
-      </c>
-      <c r="F70" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G70" s="49" t="inlineStr">
+      <c r="I70" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J70" s="49" t="inlineStr">
+        <is>
+          <t>https://toweryelectric.com/</t>
+        </is>
+      </c>
+      <c r="K70" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H70" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I70" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J70" s="49" t="inlineStr">
-        <is>
-          <t>https://eleoselectric.com/surge-protection-installation</t>
-        </is>
-      </c>
-      <c r="K70" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L70" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5355,7 +5351,7 @@
       </c>
       <c r="M70" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Advertises Type 1/Type 2 whole-home surge protection for lightning, PSPS restoration, and grid spikes across Sonoma County.</t>
+          <t>Business line: ask for Alex Towery and confirm current ownership. Dedicated Type 1/Type 2 whole-house surge-protection page, including grounding/bonding. Founded 2014; CSLB C-10 #989290. 46 Digital Dr, Ste 1.</t>
         </is>
       </c>
       <c r="N70" s="49" t="inlineStr">
@@ -5372,7 +5368,7 @@
     <row r="71" ht="48" customHeight="1" s="47">
       <c r="A71" s="49" t="inlineStr">
         <is>
-          <t>Wendt Electric Inc.</t>
+          <t>Infinium Solar, Roofing and Electric</t>
         </is>
       </c>
       <c r="B71" s="49" t="inlineStr">
@@ -5382,17 +5378,17 @@
       </c>
       <c r="C71" s="49" t="inlineStr">
         <is>
-          <t>Sebastopol, CA (Sonoma)</t>
+          <t>Campbell, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D71" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>Jeff L. (Yelp owner listing; surname not fully verified)</t>
         </is>
       </c>
       <c r="E71" s="50" t="inlineStr">
         <is>
-          <t>(707) 953-2582</t>
+          <t>(408) 583-8101</t>
         </is>
       </c>
       <c r="F71" s="49" t="inlineStr">
@@ -5400,13 +5396,11 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G71" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
+      <c r="G71" s="49" t="n">
+        <v>18</v>
       </c>
       <c r="H71" s="49" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I71" s="49" t="inlineStr">
         <is>
@@ -5415,12 +5409,12 @@
       </c>
       <c r="J71" s="49" t="inlineStr">
         <is>
-          <t>https://wendtelectric68.com/surge-protection/</t>
+          <t>https://infinium.inc/electrical/surge-protection/</t>
         </is>
       </c>
       <c r="K71" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>contact@infiniumsolar.com</t>
         </is>
       </c>
       <c r="L71" s="49" t="inlineStr">
@@ -5430,7 +5424,7 @@
       </c>
       <c r="M71" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Advertises whole-house and commercial surge protection (Leviton, Square D, Eaton). 2235 Schaeffer Rd; ~10–50 employees.</t>
+          <t>Business line: ask for Jeff and confirm current ownership. Dedicated whole-house surge-protection page. Founded 2008; CSLB #1031953. Pleasanton line (925) 401-7320. Solar/roofing/electrical contractor, not a lightning-rod specialist.</t>
         </is>
       </c>
       <c r="N71" s="49" t="inlineStr">
@@ -5447,7 +5441,7 @@
     <row r="72" ht="48" customHeight="1" s="47">
       <c r="A72" s="49" t="inlineStr">
         <is>
-          <t>YKCA Electric</t>
+          <t>Guerreros Electric, Inc.</t>
         </is>
       </c>
       <c r="B72" s="49" t="inlineStr">
@@ -5457,34 +5451,32 @@
       </c>
       <c r="C72" s="49" t="inlineStr">
         <is>
-          <t>San Carlos, CA (San Mateo)</t>
+          <t>Berkeley, CA (Alameda)</t>
         </is>
       </c>
       <c r="D72" s="49" t="inlineStr">
         <is>
+          <t>Juan Carlos Guerrero</t>
+        </is>
+      </c>
+      <c r="E72" s="50" t="inlineStr">
+        <is>
+          <t>(510) 409-3627</t>
+        </is>
+      </c>
+      <c r="F72" s="49" t="inlineStr">
+        <is>
+          <t>Owner Direct</t>
+        </is>
+      </c>
+      <c r="G72" s="49" t="n">
+        <v>12</v>
+      </c>
+      <c r="H72" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E72" s="50" t="inlineStr">
-        <is>
-          <t>(650) 550-0819</t>
-        </is>
-      </c>
-      <c r="F72" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G72" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H72" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I72" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5492,12 +5484,12 @@
       </c>
       <c r="J72" s="49" t="inlineStr">
         <is>
-          <t>https://ykca.com/</t>
+          <t>https://www.guerreroselectric.com/surge-protection</t>
         </is>
       </c>
       <c r="K72" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>carlos@guerreroselectric.com</t>
         </is>
       </c>
       <c r="L72" s="49" t="inlineStr">
@@ -5507,7 +5499,7 @@
       </c>
       <c r="M72" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Licensed C-10 &amp; B contractor serving the Peninsula. Surge/lightning is referenced in terms; confirm they actively sell lightning/surge installs before a fit discussion.</t>
+          <t>Owner-direct contact is published for Juan Carlos Guerrero; confirm they are still the current equity owner. Dedicated full-home surge-protection page. CA corp filed 2014. 2127 6th St, Berkeley.</t>
         </is>
       </c>
       <c r="N72" s="49" t="inlineStr">
@@ -5524,7 +5516,7 @@
     <row r="73" ht="48" customHeight="1" s="47">
       <c r="A73" s="49" t="inlineStr">
         <is>
-          <t>Quality Electrical Solution (QES)</t>
+          <t>Eleos Electric (John Evans Enterprises, Inc.)</t>
         </is>
       </c>
       <c r="B73" s="49" t="inlineStr">
@@ -5534,49 +5526,47 @@
       </c>
       <c r="C73" s="49" t="inlineStr">
         <is>
-          <t>Concord, CA (Contra Costa)</t>
+          <t>Windsor, CA (Sonoma)</t>
         </is>
       </c>
       <c r="D73" s="49" t="inlineStr">
         <is>
+          <t>John Evans</t>
+        </is>
+      </c>
+      <c r="E73" s="50" t="inlineStr">
+        <is>
+          <t>(707) 837-6722</t>
+        </is>
+      </c>
+      <c r="F73" s="49" t="inlineStr">
+        <is>
+          <t>Owner Direct</t>
+        </is>
+      </c>
+      <c r="G73" s="49" t="n">
+        <v>36</v>
+      </c>
+      <c r="H73" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E73" s="50" t="inlineStr">
+      <c r="I73" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J73" s="49" t="inlineStr">
+        <is>
+          <t>https://eleoselectric.com/surge-protection-installation</t>
+        </is>
+      </c>
+      <c r="K73" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F73" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G73" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H73" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I73" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J73" s="49" t="inlineStr">
-        <is>
-          <t>https://www.go-qes.com/service-areas/concord-electrical-services</t>
-        </is>
-      </c>
-      <c r="K73" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L73" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5584,7 +5574,7 @@
       </c>
       <c r="M73" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Licensed C-10 serving Concord/Hwy 4–I-680; commercial and residential electrical. Confirm explicit surge/lightning-protection offering and a published phone on the call.</t>
+          <t>Owner-direct: site says the owner usually answers; confirm John Evans is still the current equity owner. Type 1/Type 2 whole-home SPDs for lightning, PSPS, and grid spikes. CSLB #1009044. 930 Shiloh Rd, Bldg 41, Ste C.</t>
         </is>
       </c>
       <c r="N73" s="49" t="inlineStr">
@@ -5601,7 +5591,7 @@
     <row r="74" ht="48" customHeight="1" s="47">
       <c r="A74" s="49" t="inlineStr">
         <is>
-          <t>Ongaro &amp; Sons</t>
+          <t>Skyline Electric LLC</t>
         </is>
       </c>
       <c r="B74" s="49" t="inlineStr">
@@ -5611,49 +5601,47 @@
       </c>
       <c r="C74" s="49" t="inlineStr">
         <is>
-          <t>Napa / North Bay, CA</t>
+          <t>Hayward, CA (Alameda)</t>
         </is>
       </c>
       <c r="D74" s="49" t="inlineStr">
         <is>
-          <t>Ongaro family</t>
+          <t>Eduard Sandulyak</t>
         </is>
       </c>
       <c r="E74" s="50" t="inlineStr">
         <is>
-          <t>(415) 741-2820</t>
+          <t>(510) 470-0520</t>
         </is>
       </c>
       <c r="F74" s="49" t="inlineStr">
         <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G74" s="49" t="inlineStr">
+          <t>Owner Direct</t>
+        </is>
+      </c>
+      <c r="G74" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="H74" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H74" s="49" t="inlineStr">
+      <c r="I74" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J74" s="49" t="inlineStr">
+        <is>
+          <t>https://www.skylineelectricusa.com/whole-house-surge-protection</t>
+        </is>
+      </c>
+      <c r="K74" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="I74" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J74" s="49" t="inlineStr">
-        <is>
-          <t>https://ongaroandsons.com/service-area/napa-ca/</t>
-        </is>
-      </c>
-      <c r="K74" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L74" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5661,7 +5649,7 @@
       </c>
       <c r="M74" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the Ongaro family and confirm current ownership. Licensed electrical (plus HVAC/plumbing) serving Napa. Confirm they install surge/lightning-protection systems, not only general electrical.</t>
+          <t>Owner-direct contact is published for Eduard Sandulyak; confirm they are still the current equity owner. Whole-house surge plus grounding/bonding. LLC filed 2023; CSLB C-10 #1121036. 22263 Prospect St. Screening: public entity is about 3 years old.</t>
         </is>
       </c>
       <c r="N74" s="49" t="inlineStr">
@@ -5678,7 +5666,7 @@
     <row r="75" ht="48" customHeight="1" s="47">
       <c r="A75" s="49" t="inlineStr">
         <is>
-          <t>J&amp;J Electric, Inc.</t>
+          <t>Avant Electric, Inc.</t>
         </is>
       </c>
       <c r="B75" s="49" t="inlineStr">
@@ -5688,34 +5676,32 @@
       </c>
       <c r="C75" s="49" t="inlineStr">
         <is>
-          <t>Santa Rosa, CA (Sonoma)</t>
+          <t>Santa Clara, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D75" s="49" t="inlineStr">
         <is>
+          <t>Brian Gerlach (owner; firm also described as woman-owned)</t>
+        </is>
+      </c>
+      <c r="E75" s="50" t="inlineStr">
+        <is>
+          <t>(408) 688-1546</t>
+        </is>
+      </c>
+      <c r="F75" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G75" s="49" t="n">
+        <v>35</v>
+      </c>
+      <c r="H75" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E75" s="50" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="F75" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G75" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H75" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I75" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5723,12 +5709,12 @@
       </c>
       <c r="J75" s="49" t="inlineStr">
         <is>
-          <t>https://jjelectricco.com/</t>
+          <t>https://avant-electric.com/electrician/ground-wire-installation/</t>
         </is>
       </c>
       <c r="K75" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>avant@avant-electric.com</t>
         </is>
       </c>
       <c r="L75" s="49" t="inlineStr">
@@ -5738,7 +5724,7 @@
       </c>
       <c r="M75" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. C-10 contractor for Sonoma, Napa, and Marin residential/commercial electrical. Confirm surge/lightning-protection offering and published phone on the call.</t>
+          <t>Business line: ask for Brian Gerlach and confirm current ownership. Explicit grounding-system and whole-home surge pages. 2066 A Walsh Ave. Diamond Certified owner line (408) 874-6906.</t>
         </is>
       </c>
       <c r="N75" s="49" t="inlineStr">
@@ -5755,7 +5741,7 @@
     <row r="76" ht="48" customHeight="1" s="47">
       <c r="A76" s="49" t="inlineStr">
         <is>
-          <t>Wilson Electric</t>
+          <t>Dollens Electric Corporation</t>
         </is>
       </c>
       <c r="B76" s="49" t="inlineStr">
@@ -5765,49 +5751,47 @@
       </c>
       <c r="C76" s="49" t="inlineStr">
         <is>
-          <t>San Mateo / Santa Cruz / Santa Clara counties, CA</t>
+          <t>San Jose, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D76" s="49" t="inlineStr">
         <is>
+          <t>Jason Dollens (President); Josephine Dollens also listed on BBB</t>
+        </is>
+      </c>
+      <c r="E76" s="50" t="inlineStr">
+        <is>
+          <t>(408) 929-6100</t>
+        </is>
+      </c>
+      <c r="F76" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G76" s="49" t="n">
+        <v>21</v>
+      </c>
+      <c r="H76" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E76" s="50" t="inlineStr">
-        <is>
-          <t>(888) 967-5791</t>
-        </is>
-      </c>
-      <c r="F76" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G76" s="49" t="inlineStr">
+      <c r="I76" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J76" s="49" t="inlineStr">
+        <is>
+          <t>https://dollenselectric.com/whole-house-surge-protector-installation/</t>
+        </is>
+      </c>
+      <c r="K76" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H76" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I76" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J76" s="49" t="inlineStr">
-        <is>
-          <t>https://wilsonelectric.works/</t>
-        </is>
-      </c>
-      <c r="K76" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L76" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5815,7 +5799,7 @@
       </c>
       <c r="M76" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Bay Area residential electrical contractor. Confirm they actively sell surge or lightning-protection systems versus general wiring only.</t>
+          <t>Business line: ask for Jason Dollens and confirm current ownership. Dedicated San Jose whole-house surge-protector page. Family-owned; BBB founding 2004. 3240 S White Rd.</t>
         </is>
       </c>
       <c r="N76" s="49" t="inlineStr">
@@ -5832,7 +5816,7 @@
     <row r="77" ht="48" customHeight="1" s="47">
       <c r="A77" s="49" t="inlineStr">
         <is>
-          <t>JJC Electric</t>
+          <t>Arsen Electric Inc.</t>
         </is>
       </c>
       <c r="B77" s="49" t="inlineStr">
@@ -5842,49 +5826,47 @@
       </c>
       <c r="C77" s="49" t="inlineStr">
         <is>
-          <t>Fremont, CA (Alameda)</t>
+          <t>San Jose / Sunnyvale, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D77" s="49" t="inlineStr">
         <is>
+          <t>Dmitry Druzhina</t>
+        </is>
+      </c>
+      <c r="E77" s="50" t="inlineStr">
+        <is>
+          <t>(408) 594-9770</t>
+        </is>
+      </c>
+      <c r="F77" s="49" t="inlineStr">
+        <is>
+          <t>Owner Direct</t>
+        </is>
+      </c>
+      <c r="G77" s="49" t="n">
+        <v>9</v>
+      </c>
+      <c r="H77" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E77" s="50" t="inlineStr">
-        <is>
-          <t>(866) 740-1093</t>
-        </is>
-      </c>
-      <c r="F77" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G77" s="49" t="inlineStr">
+      <c r="I77" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J77" s="49" t="inlineStr">
+        <is>
+          <t>https://arsenelectric.com/</t>
+        </is>
+      </c>
+      <c r="K77" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H77" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I77" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J77" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K77" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L77" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5892,7 +5874,7 @@
       </c>
       <c r="M77" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Public listings describe a Fremont electrician offering whole-house surge protection. Verify legal name, website, and that this is not a lead-gen listing.</t>
+          <t>Owner-direct contact is published for Dmitry Druzhina; confirm they are still the current equity owner. Lists surge protection among core services. Serving Bay Area since 2017; CSLB #1034404.</t>
         </is>
       </c>
       <c r="N77" s="49" t="inlineStr">
@@ -5909,7 +5891,7 @@
     <row r="78" ht="48" customHeight="1" s="47">
       <c r="A78" s="49" t="inlineStr">
         <is>
-          <t>SFE Electric Inc.</t>
+          <t>Rocky Hill Electric Inc.</t>
         </is>
       </c>
       <c r="B78" s="49" t="inlineStr">
@@ -5919,47 +5901,45 @@
       </c>
       <c r="C78" s="49" t="inlineStr">
         <is>
-          <t>Concord, CA (Contra Costa)</t>
+          <t>San Rafael, CA (Marin)</t>
         </is>
       </c>
       <c r="D78" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified (family-owned; CEO listed on LinkedIn)</t>
+          <t>Bengiamino (Ben) E. Ielmorini</t>
         </is>
       </c>
       <c r="E78" s="50" t="inlineStr">
         <is>
+          <t>(415) 523-5201</t>
+        </is>
+      </c>
+      <c r="F78" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G78" s="49" t="n">
+        <v>7</v>
+      </c>
+      <c r="H78" s="49" t="n">
+        <v>7</v>
+      </c>
+      <c r="I78" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J78" s="49" t="inlineStr">
+        <is>
+          <t>https://www.rockyhillelectric.com/home-surge-protection-in-san-rafael-ca-why-every-modern-home-needs-it/</t>
+        </is>
+      </c>
+      <c r="K78" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F78" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G78" s="49" t="n">
-        <v>10</v>
-      </c>
-      <c r="H78" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I78" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J78" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K78" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L78" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -5967,7 +5947,7 @@
       </c>
       <c r="M78" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner/CEO. Family-owned East Bay electrical firm (panel upgrades, commercial/residential). Confirm surge/lightning offering and a working business line.</t>
+          <t>Business line: ask for Ben Ielmorini and confirm current ownership. Explicit Type 1/Type 2 panel SPD and grounding/bonding content. Founded 2019. 4330 Redwood Hwy, Ste 200. Owner has described a 7-technician team.</t>
         </is>
       </c>
       <c r="N78" s="49" t="inlineStr">
@@ -5984,7 +5964,7 @@
     <row r="79" ht="48" customHeight="1" s="47">
       <c r="A79" s="49" t="inlineStr">
         <is>
-          <t>VFC Lightning Protection — California / Western region</t>
+          <t>Divine Electric and Plumbing</t>
         </is>
       </c>
       <c r="B79" s="49" t="inlineStr">
@@ -5994,45 +5974,45 @@
       </c>
       <c r="C79" s="49" t="inlineStr">
         <is>
-          <t>Serves Bay Area projects; CA division in Ontario (SoCal)</t>
+          <t>San Rafael, CA (Marin)</t>
         </is>
       </c>
       <c r="D79" s="49" t="inlineStr">
         <is>
+          <t>Darin Divine</t>
+        </is>
+      </c>
+      <c r="E79" s="50" t="inlineStr">
+        <is>
+          <t>(415) 213-4972</t>
+        </is>
+      </c>
+      <c r="F79" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G79" s="49" t="n">
+        <v>23</v>
+      </c>
+      <c r="H79" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="I79" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J79" s="49" t="inlineStr">
+        <is>
+          <t>https://www.calldivine.com/electrical-services/home-surge-protection/</t>
+        </is>
+      </c>
+      <c r="K79" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E79" s="50" t="inlineStr">
-        <is>
-          <t>(800) 825-1948</t>
-        </is>
-      </c>
-      <c r="F79" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G79" s="49" t="n">
-        <v>37</v>
-      </c>
-      <c r="H79" s="49" t="n">
-        <v>45</v>
-      </c>
-      <c r="I79" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J79" s="49" t="inlineStr">
-        <is>
-          <t>https://vfclp.com/</t>
-        </is>
-      </c>
-      <c r="K79" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L79" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -6040,7 +6020,7 @@
       </c>
       <c r="M79" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the Western regional manager. Pure-play LPI lightning-protection contractor (est. ~1989) that staffs Bay Area projects. Confirm a local decision-maker; HQ is North Salt Lake, UT.</t>
+          <t>Business line: ask for Darin Divine and confirm current ownership. Dedicated Marin whole-house surge-protection page. Founded 2003; CSLB #817357 (C-10/C-36). 2935 Kerner Blvd, Ste E.</t>
         </is>
       </c>
       <c r="N79" s="49" t="inlineStr">
@@ -6057,7 +6037,7 @@
     <row r="80" ht="48" customHeight="1" s="47">
       <c r="A80" s="49" t="inlineStr">
         <is>
-          <t>Kuefler Lightning Protection (distributor)</t>
+          <t>Owens Electric &amp; Solar</t>
         </is>
       </c>
       <c r="B80" s="49" t="inlineStr">
@@ -6067,49 +6047,45 @@
       </c>
       <c r="C80" s="49" t="inlineStr">
         <is>
-          <t>Serves California statewide</t>
+          <t>San Mateo, CA (San Mateo)</t>
         </is>
       </c>
       <c r="D80" s="49" t="inlineStr">
         <is>
+          <t>Jeff Owens</t>
+        </is>
+      </c>
+      <c r="E80" s="50" t="inlineStr">
+        <is>
+          <t>(650) 348-5727</t>
+        </is>
+      </c>
+      <c r="F80" s="49" t="inlineStr">
+        <is>
+          <t>Owner Direct</t>
+        </is>
+      </c>
+      <c r="G80" s="49" t="n">
+        <v>61</v>
+      </c>
+      <c r="H80" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="I80" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J80" s="49" t="inlineStr">
+        <is>
+          <t>https://www.owenselectricinc.com/electrical/surge-protection</t>
+        </is>
+      </c>
+      <c r="K80" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E80" s="50" t="inlineStr">
-        <is>
-          <t>(800) 370-5886</t>
-        </is>
-      </c>
-      <c r="F80" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G80" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H80" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I80" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J80" s="49" t="inlineStr">
-        <is>
-          <t>https://kuefler-lightning.com/states/california/</t>
-        </is>
-      </c>
-      <c r="K80" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L80" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -6117,7 +6093,7 @@
       </c>
       <c r="M80" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the California sales contact. UL-listed lightning-protection materials distributor (UL 96A / NFPA 780 / LPI-175). Adjacent supplier, not a local installer — useful for installer referrals.</t>
+          <t>Owner-direct contact is published for Jeff Owens; confirm they are still the current equity owner. Dedicated residential and commercial surge-protection page, including lightning-caused surges. Family-owned since 1965; CSLB #464389. 279 N Amphlett Blvd.</t>
         </is>
       </c>
       <c r="N80" s="49" t="inlineStr">
@@ -6134,7 +6110,7 @@
     <row r="81" ht="48" customHeight="1" s="47">
       <c r="A81" s="49" t="inlineStr">
         <is>
-          <t>Bonded Lightning Protection (national specialist)</t>
+          <t>Mr. Prime Electrical</t>
         </is>
       </c>
       <c r="B81" s="49" t="inlineStr">
@@ -6144,17 +6120,17 @@
       </c>
       <c r="C81" s="49" t="inlineStr">
         <is>
-          <t>Serves CA projects; HQ Jupiter, FL</t>
+          <t>Burlingame, CA (San Mateo)</t>
         </is>
       </c>
       <c r="D81" s="49" t="inlineStr">
         <is>
-          <t>Dillon family</t>
+          <t>Jeff Balich (acquired from founder Martin Balich)</t>
         </is>
       </c>
       <c r="E81" s="50" t="inlineStr">
         <is>
-          <t>(561) 746-4336</t>
+          <t>(650) 727-3156</t>
         </is>
       </c>
       <c r="F81" s="49" t="inlineStr">
@@ -6163,7 +6139,7 @@
         </is>
       </c>
       <c r="G81" s="49" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H81" s="49" t="inlineStr">
         <is>
@@ -6177,7 +6153,7 @@
       </c>
       <c r="J81" s="49" t="inlineStr">
         <is>
-          <t>https://bondedlightning.com/</t>
+          <t>https://mrprimeelectrical.com/</t>
         </is>
       </c>
       <c r="K81" s="49" t="inlineStr">
@@ -6192,7 +6168,7 @@
       </c>
       <c r="M81" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current principal. Pure-play lightning-protection contractor (family-owned). Confirm whether they currently bid Bay Area work before a local-owner conversation.</t>
+          <t>Business line: ask for Jeff Balich and confirm current ownership. Homepage advertises whole-home surge protection. License issued 1970; current owner acquired 1995. CSLB C-10 #264901. 511 Burlingame Ave. Distinct from Mr. Electric of San Jose on the prior list.</t>
         </is>
       </c>
       <c r="N81" s="49" t="inlineStr">
@@ -6209,7 +6185,7 @@
     <row r="82" ht="48" customHeight="1" s="47">
       <c r="A82" s="49" t="inlineStr">
         <is>
-          <t>Myers Container Management Services</t>
+          <t>Container Management Services, LLC (Myers Container)</t>
         </is>
       </c>
       <c r="B82" s="49" t="inlineStr">
@@ -6224,29 +6200,29 @@
       </c>
       <c r="D82" s="49" t="inlineStr">
         <is>
+          <t>Kyle Stavig (CEO, Myers Container / Stavig family)</t>
+        </is>
+      </c>
+      <c r="E82" s="50" t="inlineStr">
+        <is>
+          <t>(800) 406-9377</t>
+        </is>
+      </c>
+      <c r="F82" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G82" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E82" s="50" t="inlineStr">
-        <is>
-          <t>(800) 406-9377</t>
-        </is>
-      </c>
-      <c r="F82" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G82" s="49" t="inlineStr">
+      <c r="H82" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H82" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I82" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6254,12 +6230,12 @@
       </c>
       <c r="J82" s="49" t="inlineStr">
         <is>
-          <t>https://resource.stopwaste.org/vendor/myers-container-management-services-hayward-21301-cloud-way</t>
+          <t>https://myerscontainer.com/</t>
         </is>
       </c>
       <c r="K82" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>jrodriguez@myerscontainer.com</t>
         </is>
       </c>
       <c r="L82" s="49" t="inlineStr">
@@ -6269,7 +6245,7 @@
       </c>
       <c r="M82" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the Hayward plant manager and confirm current ownership. Direct metal/plastic drum and barrel reconditioning and recycling. 21301 Cloud Way, Hayward, CA 94545.</t>
+          <t>Business line: ask for Kyle Stavig or Hayward ops (Joe Gresenz) and confirm current ownership. Strongest local drum fit: EPA inventory lists Myers CMS at 21301 Cloud Way as an open drum reconditioner. Metal/plastic drum and barrel reconditioning and recycling.</t>
         </is>
       </c>
       <c r="N82" s="49" t="inlineStr">
@@ -6286,7 +6262,7 @@
     <row r="83" ht="48" customHeight="1" s="47">
       <c r="A83" s="49" t="inlineStr">
         <is>
-          <t>IBC Tanks Recycling</t>
+          <t>Containers Unlimited (The Cary Company)</t>
         </is>
       </c>
       <c r="B83" s="49" t="inlineStr">
@@ -6296,34 +6272,32 @@
       </c>
       <c r="C83" s="49" t="inlineStr">
         <is>
-          <t>Hayward, CA (Alameda)</t>
+          <t>Livermore, CA (Alameda); historically Hayward/Oakland</t>
         </is>
       </c>
       <c r="D83" s="49" t="inlineStr">
         <is>
+          <t>Mike McGuire (former owner; stayed as regional VP after 2021 Cary sale)</t>
+        </is>
+      </c>
+      <c r="E83" s="50" t="inlineStr">
+        <is>
+          <t>(510) 887-9277</t>
+        </is>
+      </c>
+      <c r="F83" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G83" s="49" t="n">
+        <v>43</v>
+      </c>
+      <c r="H83" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E83" s="50" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="F83" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G83" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H83" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I83" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6331,12 +6305,12 @@
       </c>
       <c r="J83" s="49" t="inlineStr">
         <is>
-          <t>https://www.ibctanksrecycling.com/</t>
+          <t>https://containersunlimited.com/</t>
         </is>
       </c>
       <c r="K83" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>cu@thecarycompany.com</t>
         </is>
       </c>
       <c r="L83" s="49" t="inlineStr">
@@ -6346,7 +6320,7 @@
       </c>
       <c r="M83" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Hayward facility buys, sells, steam-cleans, and reconditions IBC totes (FDA-compliant washes). Verify a published phone and legal entity on the call.</t>
+          <t>Business line: ask for Mike McGuire and confirm current local decision rights. Founded 1983; drums, pails, and IBCs. Livermore is the current distribution/regional office; dedicated reconditioning plant is in Jurupa Valley. StopWaste still lists Hayward take-back.</t>
         </is>
       </c>
       <c r="N83" s="49" t="inlineStr">
@@ -6363,7 +6337,7 @@
     <row r="84" ht="48" customHeight="1" s="47">
       <c r="A84" s="49" t="inlineStr">
         <is>
-          <t>Container Technology, Inc. / IBC Recon Services — Hayward</t>
+          <t>National Tank Services (Trimac) — Hayward wash</t>
         </is>
       </c>
       <c r="B84" s="49" t="inlineStr">
@@ -6378,12 +6352,12 @@
       </c>
       <c r="D84" s="49" t="inlineStr">
         <is>
-          <t>J. Jesus Miramontes (Hayward Plant Manager)</t>
+          <t>Not publicly verified (Trimac Transportation trade name)</t>
         </is>
       </c>
       <c r="E84" s="50" t="inlineStr">
         <is>
-          <t>(800) 295-5510</t>
+          <t>(510) 972-9331</t>
         </is>
       </c>
       <c r="F84" s="49" t="inlineStr">
@@ -6408,7 +6382,7 @@
       </c>
       <c r="J84" s="49" t="inlineStr">
         <is>
-          <t>https://www.containertechnology.com/locations</t>
+          <t>https://www.nationaltankservices.com/</t>
         </is>
       </c>
       <c r="K84" s="49" t="inlineStr">
@@ -6423,7 +6397,7 @@
       </c>
       <c r="M84" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for J. Jesus Miramontes and confirm local P&amp;L ownership (corporate HQ Las Vegas). IBC reconditioning/cleaning warehouse in Hayward; also (509) 851-3117 quote line.</t>
+          <t>Business line: ask for the Hayward washrack manager. Confirmed tank-trailer wash at 3751 Breakwater Ave. Washrack also (510) 293-6838. Distinct from Quala/HTI/DCI. Hayward menu is chemical/latex tank-trailer wash; tote/IBC is a company-wide offering at other shops.</t>
         </is>
       </c>
       <c r="N84" s="49" t="inlineStr">
@@ -6440,7 +6414,7 @@
     <row r="85" ht="48" customHeight="1" s="47">
       <c r="A85" s="49" t="inlineStr">
         <is>
-          <t>Kleen Industrial Services, Inc.</t>
+          <t>ACTenviro (Advanced Chemical Transport)</t>
         </is>
       </c>
       <c r="B85" s="49" t="inlineStr">
@@ -6450,34 +6424,32 @@
       </c>
       <c r="C85" s="49" t="inlineStr">
         <is>
-          <t>Danville, CA (Contra Costa)</t>
+          <t>San Jose, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D85" s="49" t="inlineStr">
         <is>
+          <t>Not publicly verified (Republic Services parent; Tim Smith listed as CEO)</t>
+        </is>
+      </c>
+      <c r="E85" s="50" t="inlineStr">
+        <is>
+          <t>(408) 548-5050</t>
+        </is>
+      </c>
+      <c r="F85" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G85" s="49" t="n">
+        <v>26</v>
+      </c>
+      <c r="H85" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E85" s="50" t="inlineStr">
-        <is>
-          <t>(925) 831-9802</t>
-        </is>
-      </c>
-      <c r="F85" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G85" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H85" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I85" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6485,12 +6457,12 @@
       </c>
       <c r="J85" s="49" t="inlineStr">
         <is>
-          <t>https://www.kleenindustrialservices.com/</t>
+          <t>https://www.actenviro.com/</t>
         </is>
       </c>
       <c r="K85" s="49" t="inlineStr">
         <is>
-          <t>info@kleenindustrialservices.com</t>
+          <t>info@actenviro.com</t>
         </is>
       </c>
       <c r="L85" s="49" t="inlineStr">
@@ -6500,7 +6472,7 @@
       </c>
       <c r="M85" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Hazardous/non-hazardous drum removal, vacuum-truck, and industrial-waste services. 50 Oak Court, Danville. Also (800) 356-7323 / (925) 831-9183.</t>
+          <t>Business line: ask for the San Jose branch manager. Founded 2000. 967 Mabury Rd. Storage-tank steam-cleaning, UST cleaning, portable-tank cleaning, and vacuum-truck work. Adjacent industrial tank cleaning, not a drum-reconditioning plant. Emergency (866) 348-2800.</t>
         </is>
       </c>
       <c r="N85" s="49" t="inlineStr">
@@ -6517,7 +6489,7 @@
     <row r="86" ht="48" customHeight="1" s="47">
       <c r="A86" s="49" t="inlineStr">
         <is>
-          <t>Heritage-Crystal Clean — Hayward / Oakland branch</t>
+          <t>Patriot Environmental Services — Richmond</t>
         </is>
       </c>
       <c r="B86" s="49" t="inlineStr">
@@ -6527,17 +6499,17 @@
       </c>
       <c r="C86" s="49" t="inlineStr">
         <is>
-          <t>Hayward, CA (Alameda)</t>
+          <t>Richmond, CA (Contra Costa)</t>
         </is>
       </c>
       <c r="D86" s="49" t="inlineStr">
         <is>
-          <t>Corporate branch; local owner not applicable</t>
+          <t>Kent Bartley (CEO) / Josh Teves (President); Tom Salazar (Richmond Operations Manager)</t>
         </is>
       </c>
       <c r="E86" s="50" t="inlineStr">
         <is>
-          <t>(877) 938-7948</t>
+          <t>(800) 624-9136</t>
         </is>
       </c>
       <c r="F86" s="49" t="inlineStr">
@@ -6545,8 +6517,10 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G86" s="49" t="n">
-        <v>27</v>
+      <c r="G86" s="49" t="inlineStr">
+        <is>
+          <t>Not publicly verified</t>
+        </is>
       </c>
       <c r="H86" s="49" t="inlineStr">
         <is>
@@ -6560,12 +6534,12 @@
       </c>
       <c r="J86" s="49" t="inlineStr">
         <is>
-          <t>https://www.crystal-clean.com/stores/environmental-services-branch-oakland-california/</t>
+          <t>https://www.patriotenvironmental.com/locations/</t>
         </is>
       </c>
       <c r="K86" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>contact@patriotenv.com</t>
         </is>
       </c>
       <c r="L86" s="49" t="inlineStr">
@@ -6575,7 +6549,7 @@
       </c>
       <c r="M86" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the Hayward branch manager. Waste-drum disposal, parts cleaners, and used-oil services. 23271 Eichler St, Bldg 10. National platform — confirm local decision rights.</t>
+          <t>Business line: ask for Tom Salazar and confirm local decision rights (Heritage-Crystal Clean subsidiary since 2022). Hydroblasting, tank/vessel cleaning, vacuum work. 255 Parr Blvd. 24-hr dispatch (855) 666-4299.</t>
         </is>
       </c>
       <c r="N86" s="49" t="inlineStr">
@@ -6592,7 +6566,7 @@
     <row r="87" ht="48" customHeight="1" s="47">
       <c r="A87" s="49" t="inlineStr">
         <is>
-          <t>CAL INC</t>
+          <t>Clean Harbors — Benicia Industrial Services</t>
         </is>
       </c>
       <c r="B87" s="49" t="inlineStr">
@@ -6602,49 +6576,47 @@
       </c>
       <c r="C87" s="49" t="inlineStr">
         <is>
-          <t>Vacaville, CA (Solano)</t>
+          <t>Benicia, CA (Solano)</t>
         </is>
       </c>
       <c r="D87" s="49" t="inlineStr">
         <is>
+          <t>Alan S. McKim (Chairman/CTO; public company)</t>
+        </is>
+      </c>
+      <c r="E87" s="50" t="inlineStr">
+        <is>
+          <t>(707) 747-6699</t>
+        </is>
+      </c>
+      <c r="F87" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G87" s="49" t="n">
+        <v>46</v>
+      </c>
+      <c r="H87" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E87" s="50" t="inlineStr">
-        <is>
-          <t>(800) 359-4467</t>
-        </is>
-      </c>
-      <c r="F87" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G87" s="49" t="inlineStr">
+      <c r="I87" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J87" s="49" t="inlineStr">
+        <is>
+          <t>https://www.cleanharbors.com/location/benicia-industrial-services</t>
+        </is>
+      </c>
+      <c r="K87" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H87" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I87" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J87" s="49" t="inlineStr">
-        <is>
-          <t>https://cal-inc.com/abatement/industrialcleaning.php</t>
-        </is>
-      </c>
-      <c r="K87" s="49" t="inlineStr">
-        <is>
-          <t>tesparza@cal-inc.com</t>
-        </is>
-      </c>
       <c r="L87" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -6652,7 +6624,7 @@
       </c>
       <c r="M87" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for estimating (T. Esparza) and the current owner. Industrial tank, vessel, vacuum-truck, and hydroblast cleaning across the Bay Area and Northern California.</t>
+          <t>Business line: ask for the Benicia yard manager. 4101 Industrial Way. Corporate industrial services include tank/vessel cleaning, vacuum, hydroblast/steam, and ISO/rail-car container cleaning. Confirm local wash-rack scope on the call.</t>
         </is>
       </c>
       <c r="N87" s="49" t="inlineStr">
@@ -6669,7 +6641,7 @@
     <row r="88" ht="48" customHeight="1" s="47">
       <c r="A88" s="49" t="inlineStr">
         <is>
-          <t>ADCO Services</t>
+          <t>CAL INC</t>
         </is>
       </c>
       <c r="B88" s="49" t="inlineStr">
@@ -6679,17 +6651,17 @@
       </c>
       <c r="C88" s="49" t="inlineStr">
         <is>
-          <t>Serves Antioch / Martinez / Vacaville, CA</t>
+          <t>Vacaville, CA (Solano)</t>
         </is>
       </c>
       <c r="D88" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>David Esparza (President/CEO); Sandy Esparza (co-founder/VP)</t>
         </is>
       </c>
       <c r="E88" s="50" t="inlineStr">
         <is>
-          <t>(877) 254-2326</t>
+          <t>(707) 446-7996</t>
         </is>
       </c>
       <c r="F88" s="49" t="inlineStr">
@@ -6697,15 +6669,11 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G88" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H88" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
+      <c r="G88" s="49" t="n">
+        <v>47</v>
+      </c>
+      <c r="H88" s="49" t="n">
+        <v>70</v>
       </c>
       <c r="I88" s="49" t="inlineStr">
         <is>
@@ -6714,12 +6682,12 @@
       </c>
       <c r="J88" s="49" t="inlineStr">
         <is>
-          <t>https://www.americanwastehaulers.com/hazardous-waste-disposal-california</t>
+          <t>https://cal-inc.com/</t>
         </is>
       </c>
       <c r="K88" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>desparza@cal-inc.com</t>
         </is>
       </c>
       <c r="L88" s="49" t="inlineStr">
@@ -6729,7 +6697,7 @@
       </c>
       <c r="M88" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the California operations contact. Advertises tank clean-outs and hazardous-waste disposal in East Bay/Solano cities. Confirm a Bay Area operating base versus out-of-area dispatch.</t>
+          <t>Business line: ask for David Esparza and confirm current ownership. Founded 1979. On-site tank, vessel, separator, hydroblast, and vacuum-truck cleaning across the Bay Area. Toll-free (800) 359-4467. Estimating: tesparza@cal-inc.com.</t>
         </is>
       </c>
       <c r="N88" s="49" t="inlineStr">
@@ -6746,7 +6714,7 @@
     <row r="89" ht="48" customHeight="1" s="47">
       <c r="A89" s="49" t="inlineStr">
         <is>
-          <t>Patriot Environmental Services — Richmond</t>
+          <t>Triumvirate Environmental — San Leandro</t>
         </is>
       </c>
       <c r="B89" s="49" t="inlineStr">
@@ -6756,17 +6724,17 @@
       </c>
       <c r="C89" s="49" t="inlineStr">
         <is>
-          <t>Richmond, CA (Contra Costa)</t>
+          <t>San Leandro, CA (Alameda)</t>
         </is>
       </c>
       <c r="D89" s="49" t="inlineStr">
         <is>
-          <t>Tom Salazar (Operations Manager)</t>
+          <t>John F. McQuillan (Founder/CEO/Chairman)</t>
         </is>
       </c>
       <c r="E89" s="50" t="inlineStr">
         <is>
-          <t>(800) 624-9136</t>
+          <t>(510) 447-5688</t>
         </is>
       </c>
       <c r="F89" s="49" t="inlineStr">
@@ -6774,31 +6742,29 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G89" s="49" t="inlineStr">
+      <c r="G89" s="49" t="n">
+        <v>38</v>
+      </c>
+      <c r="H89" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H89" s="49" t="inlineStr">
+      <c r="I89" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J89" s="49" t="inlineStr">
+        <is>
+          <t>https://www.triumvirate.com/locations/pacific/san-leandro-ca</t>
+        </is>
+      </c>
+      <c r="K89" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="I89" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J89" s="49" t="inlineStr">
-        <is>
-          <t>https://www.patriotenvironmental.com/locations/</t>
-        </is>
-      </c>
-      <c r="K89" s="49" t="inlineStr">
-        <is>
-          <t>contact@patriotenv.com</t>
-        </is>
-      </c>
       <c r="L89" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -6806,7 +6772,7 @@
       </c>
       <c r="M89" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for Tom Salazar and confirm local decision rights (now part of Crystal Clean). Industrial cleaning, tank/field services, and waste management. 255 Parr Blvd, Richmond, CA 94801.</t>
+          <t>Business line: ask for the San Leandro manager. 1599 Factor Ave. Location page states the facility cleans tanks; corporate pages list chemical/process tank cleaning, vacuum trucks, and confined space. Life-sciences/industrial fit, not drum reconditioning. Sales (888) 834-9697.</t>
         </is>
       </c>
       <c r="N89" s="49" t="inlineStr">
@@ -6823,7 +6789,7 @@
     <row r="90" ht="48" customHeight="1" s="47">
       <c r="A90" s="49" t="inlineStr">
         <is>
-          <t>Bayarea Terminals (ISO tank depot brand)</t>
+          <t>Golden Gate Tank Removal, Inc.</t>
         </is>
       </c>
       <c r="B90" s="49" t="inlineStr">
@@ -6833,49 +6799,45 @@
       </c>
       <c r="C90" s="49" t="inlineStr">
         <is>
-          <t>Oakland-branded ISO tank services (verify CA depot)</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="D90" s="49" t="inlineStr">
         <is>
+          <t>Tim Hallen (President; BBB). CA SOS has also listed Gina Abo Wee as CEO/CFO</t>
+        </is>
+      </c>
+      <c r="E90" s="50" t="inlineStr">
+        <is>
+          <t>(415) 512-1555</t>
+        </is>
+      </c>
+      <c r="F90" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G90" s="49" t="n">
+        <v>31</v>
+      </c>
+      <c r="H90" s="49" t="n">
+        <v>15</v>
+      </c>
+      <c r="I90" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J90" s="49" t="inlineStr">
+        <is>
+          <t>https://ggtr.com/</t>
+        </is>
+      </c>
+      <c r="K90" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E90" s="50" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="F90" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G90" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H90" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I90" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J90" s="49" t="inlineStr">
-        <is>
-          <t>https://bayareapl.com/tank-container-service/</t>
-        </is>
-      </c>
-      <c r="K90" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L90" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -6883,7 +6845,7 @@
       </c>
       <c r="M90" s="49" t="inlineStr">
         <is>
-          <t>Ask for the depot manager. Site describes Groninger automated ISO-tank and road-tanker cleaning. Corporate pages also reference India facilities — verify a live Oakland/Bay Area depot before outreach.</t>
+          <t>Business line: ask for Tim Hallen and confirm current ownership. UST cleaning, removal, and closure since 1995. CSLB #616521 (A/HAZ). 1480 Carroll Ave. Adjacent industrial tank cleaning, not drum/IBC depot work.</t>
         </is>
       </c>
       <c r="N90" s="49" t="inlineStr">
@@ -6900,7 +6862,7 @@
     <row r="91" ht="48" customHeight="1" s="47">
       <c r="A91" s="49" t="inlineStr">
         <is>
-          <t>Hoover CS — IBC / tote / ISO tank cleaning</t>
+          <t>Questar Inc. / Questar Solutions — Hayward</t>
         </is>
       </c>
       <c r="B91" s="49" t="inlineStr">
@@ -6910,49 +6872,47 @@
       </c>
       <c r="C91" s="49" t="inlineStr">
         <is>
-          <t>Serves West Coast; confirm Bay Area depot</t>
+          <t>Hayward, CA (Alameda)</t>
         </is>
       </c>
       <c r="D91" s="49" t="inlineStr">
         <is>
+          <t>Not publicly verified (Doug Rountree listed as manager on a third-party directory)</t>
+        </is>
+      </c>
+      <c r="E91" s="50" t="inlineStr">
+        <is>
+          <t>(510) 324-1333</t>
+        </is>
+      </c>
+      <c r="F91" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G91" s="49" t="n">
+        <v>36</v>
+      </c>
+      <c r="H91" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E91" s="50" t="inlineStr">
+      <c r="I91" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J91" s="49" t="inlineStr">
+        <is>
+          <t>https://www.questarsolutions.com/</t>
+        </is>
+      </c>
+      <c r="K91" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F91" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G91" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H91" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I91" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J91" s="49" t="inlineStr">
-        <is>
-          <t>https://hooversolutions.com/services/tank-cleaning-and-maintenance/</t>
-        </is>
-      </c>
-      <c r="K91" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L91" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -6960,7 +6920,7 @@
       </c>
       <c r="M91" s="49" t="inlineStr">
         <is>
-          <t>Ask for the Western/California depot contact. Certified IBC, tote, and ISO tank wash/retest. Confirm a Bay Area operating location; do not treat as a local owner-operator until verified.</t>
+          <t>Business line: ask for the Hayward yard manager. 30983 San Clemente St. StopWaste documents metal/plastic/fiber drum take-back; Questar sells new and reconditioned drums and IBC totes. Reconditioned-drum supply/take-back, not a confirmed on-site industrial wash line.</t>
         </is>
       </c>
       <c r="N91" s="49" t="inlineStr">

</xml_diff>

<commit_message>
Upgrade janitorial prospects with verified local operators
Replace thin or unverified janitorial rows with documented Bay Area firms that have published phones, websites, and principals. Refresh keeper rows with owner, email, age, and address details from public sources.

Co-authored-by: anthonyleedu <anthonyleedu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Builder + Caller Masterlist - SBC 2026.xlsx
+++ b/Builder + Caller Masterlist - SBC 2026.xlsx
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C20" s="49" t="inlineStr">
         <is>
-          <t>San Jose, CA (Santa Clara)</t>
+          <t>Santa Clara, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D20" s="49" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="K20" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>tbm@tbmfirst.net</t>
         </is>
       </c>
       <c r="L20" s="49" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="M20" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner or president. Commercial janitorial since 1986; green cleaning, window, carpet, pressure washing, and cleanroom work across Silicon Valley.</t>
+          <t>Business line: ask for the current owner or president. Commercial janitorial since 1986 at 3020 Scott Blvd; green cleaning, window, carpet, pressure washing, and cleanroom work.</t>
         </is>
       </c>
       <c r="N20" s="49" t="inlineStr">
@@ -1738,12 +1738,12 @@
       </c>
       <c r="C23" s="49" t="inlineStr">
         <is>
-          <t>Walnut Creek / East Bay, CA</t>
+          <t>Walnut Creek, CA (Contra Costa)</t>
         </is>
       </c>
       <c r="D23" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>Matthew C. Townsend</t>
         </is>
       </c>
       <c r="E23" s="50" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="K23" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@tsmaintenance.com</t>
         </is>
       </c>
       <c r="L23" s="49" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="M23" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. 25+ years of industrial, corporate, and small-business janitorial; green-cleaning programs.</t>
+          <t>Business line: ask for Matthew C. Townsend and confirm current ownership. 25+ years of industrial, corporate, and small-business janitorial. 1601 N California Blvd, Ste 250. Distinct from Tetra Maintenance.</t>
         </is>
       </c>
       <c r="N23" s="49" t="inlineStr">
@@ -1979,16 +1979,14 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G26" s="49" t="inlineStr">
+      <c r="G26" s="49" t="n">
+        <v>50</v>
+      </c>
+      <c r="H26" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H26" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I26" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2001,7 +1999,7 @@
       </c>
       <c r="K26" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@grapevinejanitorial.com</t>
         </is>
       </c>
       <c r="L26" s="49" t="inlineStr">
@@ -2011,7 +2009,7 @@
       </c>
       <c r="M26" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Commercial/industrial janitorial for offices, manufacturing, warehouses, and retail in Napa Valley. PO Box 3124.</t>
+          <t>Business line: ask for the current owner. Wine Country commercial/industrial janitorial since 1976. PO Box 3124, Napa.</t>
         </is>
       </c>
       <c r="N26" s="49" t="inlineStr">
@@ -2255,7 +2253,7 @@
     <row r="30" ht="48" customHeight="1" s="47">
       <c r="A30" s="49" t="inlineStr">
         <is>
-          <t>North Bay Building Maintenance Company</t>
+          <t>SourceONE Building Maintenance, Inc.</t>
         </is>
       </c>
       <c r="B30" s="49" t="inlineStr">
@@ -2265,7 +2263,7 @@
       </c>
       <c r="C30" s="49" t="inlineStr">
         <is>
-          <t>San Jose, CA (Santa Clara)</t>
+          <t>Santa Clara, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D30" s="49" t="inlineStr">
@@ -2275,7 +2273,7 @@
       </c>
       <c r="E30" s="50" t="inlineStr">
         <is>
-          <t>(408) 528-4238</t>
+          <t>(408) 437-3046</t>
         </is>
       </c>
       <c r="F30" s="49" t="inlineStr">
@@ -2284,7 +2282,7 @@
         </is>
       </c>
       <c r="G30" s="49" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H30" s="49" t="inlineStr">
         <is>
@@ -2293,17 +2291,17 @@
       </c>
       <c r="I30" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J30" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://www.sourceonebuildingmtn.com/</t>
         </is>
       </c>
       <c r="K30" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>jnigro@source1services.net</t>
         </is>
       </c>
       <c r="L30" s="49" t="inlineStr">
@@ -2313,7 +2311,7 @@
       </c>
       <c r="M30" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Blue Book: in business since 1999; complete janitorial and exterior building cleaning across the nine-county Bay Area.</t>
+          <t>Business line: ask for the current owner. Veteran-owned commercial janitorial for offices, labs, cleanrooms, and GMP/biotech. 2974 Scott Blvd. Public listings cite ISO 9001:2015.</t>
         </is>
       </c>
       <c r="N30" s="49" t="inlineStr">
@@ -2330,7 +2328,7 @@
     <row r="31" ht="48" customHeight="1" s="47">
       <c r="A31" s="49" t="inlineStr">
         <is>
-          <t>Maintenance Systems Management, Inc.</t>
+          <t>Altos Building Maintenance</t>
         </is>
       </c>
       <c r="B31" s="49" t="inlineStr">
@@ -2340,32 +2338,32 @@
       </c>
       <c r="C31" s="49" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Santa Clara, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D31" s="49" t="inlineStr">
         <is>
+          <t>Roger Cruickshank (Founder)</t>
+        </is>
+      </c>
+      <c r="E31" s="50" t="inlineStr">
+        <is>
+          <t>(408) 480-1630</t>
+        </is>
+      </c>
+      <c r="F31" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G31" s="49" t="n">
+        <v>38</v>
+      </c>
+      <c r="H31" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E31" s="50" t="inlineStr">
-        <is>
-          <t>(415) 920-3840</t>
-        </is>
-      </c>
-      <c r="F31" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G31" s="49" t="n">
-        <v>37</v>
-      </c>
-      <c r="H31" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I31" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2373,12 +2371,12 @@
       </c>
       <c r="J31" s="49" t="inlineStr">
         <is>
-          <t>https://msm-inc.com/</t>
+          <t>https://altosmaint.com/</t>
         </is>
       </c>
       <c r="K31" s="49" t="inlineStr">
         <is>
-          <t>sales@msm-inc.com</t>
+          <t>chase@altosmaint.com</t>
         </is>
       </c>
       <c r="L31" s="49" t="inlineStr">
@@ -2388,7 +2386,7 @@
       </c>
       <c r="M31" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the president/owner (site says owner-operated since 1989). Contract custodial for offices, schools, retail, and property managers. 2415 Third St, Ste 257.</t>
+          <t>Business line: ask for Roger Cruickshank and confirm current ownership. Founded 1988. 3080 Olcott St, Ste 105B. Serves Santa Clara, San Jose, Mountain View, and Sunnyvale.</t>
         </is>
       </c>
       <c r="N31" s="49" t="inlineStr">
@@ -2881,16 +2879,14 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G38" s="49" t="inlineStr">
+      <c r="G38" s="49" t="n">
+        <v>21</v>
+      </c>
+      <c r="H38" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H38" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I38" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2898,12 +2894,12 @@
       </c>
       <c r="J38" s="49" t="inlineStr">
         <is>
-          <t>http://www.pcsmaint.com/</t>
+          <t>https://pcsmaint.com/</t>
         </is>
       </c>
       <c r="K38" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>pcs-operations@att.net</t>
         </is>
       </c>
       <c r="L38" s="49" t="inlineStr">
@@ -2913,7 +2909,7 @@
       </c>
       <c r="M38" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. IJCSA-certified commercial/residential cleaning; 280 Newhall St, San Francisco. Also lists an LA address on the same phone.</t>
+          <t>Business line: ask for the current owner. IJCSA/BSCAI-listed commercial/residential cleaning; founded 2005. 280 Newhall St. Distinct from Professional Cleaning Systems on the prior list.</t>
         </is>
       </c>
       <c r="N38" s="49" t="inlineStr">
@@ -3335,31 +3331,29 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G44" s="49" t="inlineStr">
+      <c r="G44" s="49" t="n">
+        <v>24</v>
+      </c>
+      <c r="H44" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H44" s="49" t="inlineStr">
+      <c r="I44" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J44" s="49" t="inlineStr">
+        <is>
+          <t>https://eveningjanitorial.com/</t>
+        </is>
+      </c>
+      <c r="K44" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="I44" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J44" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K44" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L44" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -3367,7 +3361,7 @@
       </c>
       <c r="M44" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Public listings describe office and manufacturing janitorial from Walnut Creek across the East Bay. Verify website and ownership on the call.</t>
+          <t>Business line: ask for the current owner. Family-run East Bay commercial cleaning for offices, schools, and light industrial since 2002. 10 Jolie Ln. Some directories also list (925) 437-9001.</t>
         </is>
       </c>
       <c r="N44" s="49" t="inlineStr">
@@ -3384,7 +3378,7 @@
     <row r="45" ht="48" customHeight="1" s="47">
       <c r="A45" s="49" t="inlineStr">
         <is>
-          <t>ServiceMaster Janitorial by Pratik</t>
+          <t>A &amp; K Janitorial Inc.</t>
         </is>
       </c>
       <c r="B45" s="49" t="inlineStr">
@@ -3394,45 +3388,45 @@
       </c>
       <c r="C45" s="49" t="inlineStr">
         <is>
-          <t>Hayward, CA (Alameda)</t>
+          <t>San Jose, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D45" s="49" t="inlineStr">
         <is>
-          <t>Pratik (public principal; surname not displayed)</t>
+          <t>Not publicly verified</t>
         </is>
       </c>
       <c r="E45" s="50" t="inlineStr">
         <is>
+          <t>(408) 532-6889</t>
+        </is>
+      </c>
+      <c r="F45" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G45" s="49" t="n">
+        <v>33</v>
+      </c>
+      <c r="H45" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F45" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G45" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H45" s="49" t="n">
-        <v>8</v>
-      </c>
       <c r="I45" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J45" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://www.aandkjanitorial.com/</t>
         </is>
       </c>
       <c r="K45" s="49" t="inlineStr">
         <is>
-          <t>info@smjbypratik.com</t>
+          <t>jramirez@aandkjanitorial.com</t>
         </is>
       </c>
       <c r="L45" s="49" t="inlineStr">
@@ -3442,7 +3436,7 @@
       </c>
       <c r="M45" s="49" t="inlineStr">
         <is>
-          <t>Ask for Pratik and confirm current ownership. LinkedIn: Hayward HQ, 1–10 employees; disinfection and janitorial. Verify working phone during the call.</t>
+          <t>Business line: ask for the current owner. Family-owned commercial janitorial since 1993 for medical offices, schools, corporate, dealerships, and hotels.</t>
         </is>
       </c>
       <c r="N45" s="49" t="inlineStr">
@@ -3459,7 +3453,7 @@
     <row r="46" ht="48" customHeight="1" s="47">
       <c r="A46" s="49" t="inlineStr">
         <is>
-          <t>Performance First Building Services, Inc.</t>
+          <t>JP Enterprises Janitorial</t>
         </is>
       </c>
       <c r="B46" s="49" t="inlineStr">
@@ -3469,47 +3463,45 @@
       </c>
       <c r="C46" s="49" t="inlineStr">
         <is>
-          <t>Santa Clara, CA (Santa Clara)</t>
+          <t>San Mateo, CA (San Mateo)</t>
         </is>
       </c>
       <c r="D46" s="49" t="inlineStr">
         <is>
+          <t>John Velichko and Peter Velichko (Founders)</t>
+        </is>
+      </c>
+      <c r="E46" s="50" t="inlineStr">
+        <is>
+          <t>(650) 348-8991</t>
+        </is>
+      </c>
+      <c r="F46" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G46" s="49" t="n">
+        <v>40</v>
+      </c>
+      <c r="H46" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E46" s="50" t="inlineStr">
-        <is>
-          <t>(408) 441-4632</t>
-        </is>
-      </c>
-      <c r="F46" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G46" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H46" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I46" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J46" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://sanmateobestjanitorial.com/</t>
         </is>
       </c>
       <c r="K46" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>jpentrp@aol.com</t>
         </is>
       </c>
       <c r="L46" s="49" t="inlineStr">
@@ -3519,7 +3511,7 @@
       </c>
       <c r="M46" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Public directories list a Santa Clara commercial building-services firm. Website (perfirst.com) was not live at compile time; verify fit on the call.</t>
+          <t>Business line: ask for John or Peter Velichko and confirm current ownership. Peninsula janitorial since 1986. 3315 Marisma St.</t>
         </is>
       </c>
       <c r="N46" s="49" t="inlineStr">
@@ -3536,7 +3528,7 @@
     <row r="47" ht="48" customHeight="1" s="47">
       <c r="A47" s="49" t="inlineStr">
         <is>
-          <t>Apex Business Services, Inc. (Apex Construction Janitorial)</t>
+          <t>All Janitorial Service, Inc.</t>
         </is>
       </c>
       <c r="B47" s="49" t="inlineStr">
@@ -3546,47 +3538,47 @@
       </c>
       <c r="C47" s="49" t="inlineStr">
         <is>
-          <t>San Jose, CA (Santa Clara)</t>
+          <t>Redwood City, CA (San Mateo)</t>
         </is>
       </c>
       <c r="D47" s="49" t="inlineStr">
         <is>
+          <t>Christian (Chris) Ramirez (CEO)</t>
+        </is>
+      </c>
+      <c r="E47" s="50" t="inlineStr">
+        <is>
+          <t>(650) 261-0723</t>
+        </is>
+      </c>
+      <c r="F47" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G47" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E47" s="50" t="inlineStr">
+      <c r="H47" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="I47" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J47" s="49" t="inlineStr">
+        <is>
+          <t>https://www.alljanitorialservice.com/</t>
+        </is>
+      </c>
+      <c r="K47" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F47" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G47" s="49" t="n">
-        <v>41</v>
-      </c>
-      <c r="H47" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I47" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J47" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K47" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L47" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -3594,7 +3586,7 @@
       </c>
       <c r="M47" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Blue Book: established 1985; construction/finish janitorial and building maintenance in the South Bay. Verify working phone during the call.</t>
+          <t>Business line: ask for Chris Ramirez and confirm current ownership. In-house commercial janitorial, porter, floor, window, and pressure washing for San Mateo and west Santa Clara. 3130 Spring St.</t>
         </is>
       </c>
       <c r="N47" s="49" t="inlineStr">
@@ -3621,49 +3613,45 @@
       </c>
       <c r="C48" s="49" t="inlineStr">
         <is>
-          <t>Bay Area, CA</t>
+          <t>Santa Rosa, CA (Sonoma)</t>
         </is>
       </c>
       <c r="D48" s="49" t="inlineStr">
         <is>
-          <t>Adolfo Mendoza (CEO)</t>
+          <t>Adolfo Mendoza (President)</t>
         </is>
       </c>
       <c r="E48" s="50" t="inlineStr">
         <is>
+          <t>(707) 586-6640</t>
+        </is>
+      </c>
+      <c r="F48" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G48" s="49" t="n">
+        <v>47</v>
+      </c>
+      <c r="H48" s="49" t="n">
+        <v>45</v>
+      </c>
+      <c r="I48" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J48" s="49" t="inlineStr">
+        <is>
+          <t>https://optimabuildingservices.com/</t>
+        </is>
+      </c>
+      <c r="K48" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F48" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G48" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H48" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I48" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J48" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K48" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L48" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -3671,7 +3659,7 @@
       </c>
       <c r="M48" s="49" t="inlineStr">
         <is>
-          <t>Ask for Adolfo Mendoza and confirm current ownership. Public profiles describe a Bay Area commercial janitorial/facilities firm. Verify phone, city, and headcount on the call.</t>
+          <t>Business line: ask for Adolfo Mendoza and confirm current ownership. Commercial janitorial, carpet, pressure washing, and construction cleanup since 1979. BBB-accredited; about 45 employees.</t>
         </is>
       </c>
       <c r="N48" s="49" t="inlineStr">
@@ -3688,7 +3676,7 @@
     <row r="49" ht="48" customHeight="1" s="47">
       <c r="A49" s="49" t="inlineStr">
         <is>
-          <t>Redwood Building Maintenance</t>
+          <t>Redwood Building Maintenance, Inc.</t>
         </is>
       </c>
       <c r="B49" s="49" t="inlineStr">
@@ -3698,7 +3686,7 @@
       </c>
       <c r="C49" s="49" t="inlineStr">
         <is>
-          <t>East Bay / Tri-Valley, CA</t>
+          <t>Santa Rosa, CA (Sonoma); South/East Bay ops</t>
         </is>
       </c>
       <c r="D49" s="49" t="inlineStr">
@@ -3708,7 +3696,7 @@
       </c>
       <c r="E49" s="50" t="inlineStr">
         <is>
-          <t>(925) 867-3850</t>
+          <t>(888) 789-0600</t>
         </is>
       </c>
       <c r="F49" s="49" t="inlineStr">
@@ -3716,31 +3704,29 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G49" s="49" t="inlineStr">
+      <c r="G49" s="49" t="n">
+        <v>61</v>
+      </c>
+      <c r="H49" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H49" s="49" t="inlineStr">
+      <c r="I49" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J49" s="49" t="inlineStr">
+        <is>
+          <t>https://rbmco.com/</t>
+        </is>
+      </c>
+      <c r="K49" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="I49" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J49" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K49" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L49" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -3748,7 +3734,7 @@
       </c>
       <c r="M49" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Public listings place a commercial janitorial provider serving East and South Bay. Confirm legal name, city, and website on the call.</t>
+          <t>Business line: ask for the current owner. Full-service commercial janitorial since 1965. North Bay (888) 789-0600; South &amp; East Bay (925) 867-3850.</t>
         </is>
       </c>
       <c r="N49" s="49" t="inlineStr">
@@ -3765,7 +3751,7 @@
     <row r="50" ht="48" customHeight="1" s="47">
       <c r="A50" s="49" t="inlineStr">
         <is>
-          <t>Commercial Building Maintenance LLC</t>
+          <t>DSP Janitorial Service</t>
         </is>
       </c>
       <c r="B50" s="49" t="inlineStr">
@@ -3775,17 +3761,17 @@
       </c>
       <c r="C50" s="49" t="inlineStr">
         <is>
-          <t>Santa Clara, CA (Santa Clara)</t>
+          <t>Hayward, CA (Alameda)</t>
         </is>
       </c>
       <c r="D50" s="49" t="inlineStr">
         <is>
-          <t>Allen (Owner; given name not fully displayed)</t>
+          <t>Don (first name published; surname not independently verified)</t>
         </is>
       </c>
       <c r="E50" s="50" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>(510) 782-2200</t>
         </is>
       </c>
       <c r="F50" s="49" t="inlineStr">
@@ -3794,26 +3780,24 @@
         </is>
       </c>
       <c r="G50" s="49" t="n">
-        <v>5</v>
-      </c>
-      <c r="H50" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
+        <v>57</v>
+      </c>
+      <c r="H50" s="49" t="n">
+        <v>20</v>
       </c>
       <c r="I50" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J50" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://dspjanitorial.com/</t>
         </is>
       </c>
       <c r="K50" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>don@dspjanitorial.com</t>
         </is>
       </c>
       <c r="L50" s="49" t="inlineStr">
@@ -3823,7 +3807,7 @@
       </c>
       <c r="M50" s="49" t="inlineStr">
         <is>
-          <t>Ask for the owner (BBB lists Allen) and confirm current ownership. BBB: 2445 Augustine Dr #150; founded 2021. Screening concern: public evidence indicates only 5 years in business.</t>
+          <t>Business line: ask for Don and confirm current ownership. Commercial janitorial since 1969. 23762 Foley St #3. About 20 employees per BBB. Serves SF, Alameda, Santa Clara, San Mateo, and Contra Costa.</t>
         </is>
       </c>
       <c r="N50" s="49" t="inlineStr">
@@ -3840,7 +3824,7 @@
     <row r="51" ht="48" customHeight="1" s="47">
       <c r="A51" s="49" t="inlineStr">
         <is>
-          <t>Herreras Cleaning</t>
+          <t>Comet Property Services</t>
         </is>
       </c>
       <c r="B51" s="49" t="inlineStr">
@@ -3850,49 +3834,45 @@
       </c>
       <c r="C51" s="49" t="inlineStr">
         <is>
-          <t>Bay Area, CA</t>
+          <t>Novato, CA (Marin)</t>
         </is>
       </c>
       <c r="D51" s="49" t="inlineStr">
         <is>
+          <t>Richard Basile (Owner)</t>
+        </is>
+      </c>
+      <c r="E51" s="50" t="inlineStr">
+        <is>
+          <t>(415) 382-1150</t>
+        </is>
+      </c>
+      <c r="F51" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G51" s="49" t="n">
+        <v>43</v>
+      </c>
+      <c r="H51" s="49" t="n">
+        <v>110</v>
+      </c>
+      <c r="I51" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J51" s="49" t="inlineStr">
+        <is>
+          <t>https://cometps.com/</t>
+        </is>
+      </c>
+      <c r="K51" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E51" s="50" t="inlineStr">
-        <is>
-          <t>(844) 225-6243</t>
-        </is>
-      </c>
-      <c r="F51" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G51" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H51" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I51" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J51" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K51" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L51" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -3900,7 +3880,7 @@
       </c>
       <c r="M51" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Blue Book-adjacent listing for janitorial/building cleaning. Verify city, legal name, and website on the call.</t>
+          <t>Business line: ask for Richard Basile and confirm current ownership. Marin commercial contract cleaning since ~1983. 21 Commercial Blvd, Ste 12. About 110 employees per BBB. Toll-free (800) 339-1035.</t>
         </is>
       </c>
       <c r="N51" s="49" t="inlineStr">
@@ -3927,7 +3907,7 @@
       </c>
       <c r="C52" s="49" t="inlineStr">
         <is>
-          <t>Los Gatos / South Bay, CA</t>
+          <t>San Jose, CA (Santa Clara)</t>
         </is>
       </c>
       <c r="D52" s="49" t="inlineStr">
@@ -3937,24 +3917,24 @@
       </c>
       <c r="E52" s="50" t="inlineStr">
         <is>
+          <t>(408) 625-7028</t>
+        </is>
+      </c>
+      <c r="F52" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G52" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F52" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G52" s="49" t="inlineStr">
+      <c r="H52" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H52" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I52" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3967,7 +3947,7 @@
       </c>
       <c r="K52" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>abm@abmclean.com</t>
         </is>
       </c>
       <c r="L52" s="49" t="inlineStr">
@@ -3977,7 +3957,7 @@
       </c>
       <c r="M52" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Site advertises janitorial, landscaping, and facility maintenance (Los Gatos museum testimonial). Verify phone, legal entity, and HQ city — a similarly named Sacramento firm also exists.</t>
+          <t>Business line: ask for the current owner. Janitorial plus landscaping and facility maintenance. Confirm this San Jose operator versus similarly named out-of-area firms.</t>
         </is>
       </c>
       <c r="N52" s="49" t="inlineStr">
@@ -3994,7 +3974,7 @@
     <row r="53" ht="48" customHeight="1" s="47">
       <c r="A53" s="49" t="inlineStr">
         <is>
-          <t>Signature Facilities Services</t>
+          <t>Premier Janitorial SF (House Cleaning SF, LLC)</t>
         </is>
       </c>
       <c r="B53" s="49" t="inlineStr">
@@ -4004,34 +3984,32 @@
       </c>
       <c r="C53" s="49" t="inlineStr">
         <is>
-          <t>Fremont, CA (Alameda)</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="D53" s="49" t="inlineStr">
         <is>
+          <t>Noe Silva</t>
+        </is>
+      </c>
+      <c r="E53" s="50" t="inlineStr">
+        <is>
+          <t>(415) 742-1910</t>
+        </is>
+      </c>
+      <c r="F53" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G53" s="49" t="n">
+        <v>9</v>
+      </c>
+      <c r="H53" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E53" s="50" t="inlineStr">
-        <is>
-          <t>(866) 943-4588</t>
-        </is>
-      </c>
-      <c r="F53" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G53" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H53" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I53" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4039,12 +4017,12 @@
       </c>
       <c r="J53" s="49" t="inlineStr">
         <is>
-          <t>https://signaturefacilities.com/</t>
+          <t>https://housecleaningsf.com/</t>
         </is>
       </c>
       <c r="K53" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@housecleaningsf.com</t>
         </is>
       </c>
       <c r="L53" s="49" t="inlineStr">
@@ -4054,7 +4032,7 @@
       </c>
       <c r="M53" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the local principal. Public listings describe integrated janitorial/facilities work in Fremont. Confirm whether this is an independent Bay Area shop versus a national brand office.</t>
+          <t>Business line: ask for Noe Silva and confirm current ownership. Diamond Certified commercial janitorial division. Distinct from Premier Commercial Cleaning Solutions on the prior list.</t>
         </is>
       </c>
       <c r="N53" s="49" t="inlineStr">
@@ -4071,7 +4049,7 @@
     <row r="54" ht="48" customHeight="1" s="47">
       <c r="A54" s="49" t="inlineStr">
         <is>
-          <t>Jani-King of the San Francisco Bay Area</t>
+          <t>Enviro-Master of North Bay</t>
         </is>
       </c>
       <c r="B54" s="49" t="inlineStr">
@@ -4081,49 +4059,49 @@
       </c>
       <c r="C54" s="49" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area, CA</t>
+          <t>Novato, CA (Marin)</t>
         </is>
       </c>
       <c r="D54" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified (regional franchise)</t>
+          <t>Ash Gorringe (Owner)</t>
         </is>
       </c>
       <c r="E54" s="50" t="inlineStr">
         <is>
+          <t>(415) 200-2638</t>
+        </is>
+      </c>
+      <c r="F54" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G54" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F54" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G54" s="49" t="inlineStr">
+      <c r="H54" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H54" s="49" t="inlineStr">
+      <c r="I54" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J54" s="49" t="inlineStr">
+        <is>
+          <t>https://california.enviro-master.com/commercial-cleaning-locations/north-bay/</t>
+        </is>
+      </c>
+      <c r="K54" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="I54" s="49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J54" s="49" t="inlineStr">
-        <is>
-          <t>https://www.janiking.com/</t>
-        </is>
-      </c>
-      <c r="K54" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L54" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -4131,7 +4109,7 @@
       </c>
       <c r="M54" s="49" t="inlineStr">
         <is>
-          <t>Ask for the regional/franchise owner. National commercial-cleaning franchise with Bay Area operators. Verify local office phone, city, and owner on the call.</t>
+          <t>Business line: ask for Ash Gorringe and confirm current ownership. North Bay franchise for restroom/hygiene, janitorial supplies, windows, and commercial cleaning. 74 Digital Dr.</t>
         </is>
       </c>
       <c r="N54" s="49" t="inlineStr">
@@ -4225,7 +4203,7 @@
     <row r="56" ht="48" customHeight="1" s="47">
       <c r="A56" s="49" t="inlineStr">
         <is>
-          <t>Building Maintenance Solutions, Inc.</t>
+          <t>Alford Janitorial Services, LLC</t>
         </is>
       </c>
       <c r="B56" s="49" t="inlineStr">
@@ -4235,7 +4213,7 @@
       </c>
       <c r="C56" s="49" t="inlineStr">
         <is>
-          <t>Pittsburg, CA (Contra Costa)</t>
+          <t>Concord, CA (Contra Costa)</t>
         </is>
       </c>
       <c r="D56" s="49" t="inlineStr">
@@ -4245,37 +4223,37 @@
       </c>
       <c r="E56" s="50" t="inlineStr">
         <is>
+          <t>(510) 943-8752</t>
+        </is>
+      </c>
+      <c r="F56" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G56" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F56" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G56" s="49" t="inlineStr">
+      <c r="H56" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H56" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I56" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J56" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://alfordjanitorial.com/</t>
         </is>
       </c>
       <c r="K56" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@alfordjanitorial.com</t>
         </is>
       </c>
       <c r="L56" s="49" t="inlineStr">
@@ -4285,7 +4263,7 @@
       </c>
       <c r="M56" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Public directories list a Pittsburg-area commercial janitorial firm. Verify phone, website, and ownership on the call.</t>
+          <t>Business line: ask for the current owner. Family-owned East Bay commercial janitorial for offices, schools, churches, clinics, gyms, and retail. 1265 Pine Creek Wy.</t>
         </is>
       </c>
       <c r="N56" s="49" t="inlineStr">
@@ -4302,7 +4280,7 @@
     <row r="57" ht="48" customHeight="1" s="47">
       <c r="A57" s="49" t="inlineStr">
         <is>
-          <t>Classic Janitorial Service</t>
+          <t>GDL Building Maintenance</t>
         </is>
       </c>
       <c r="B57" s="49" t="inlineStr">
@@ -4312,7 +4290,7 @@
       </c>
       <c r="C57" s="49" t="inlineStr">
         <is>
-          <t>Hayward, CA (Alameda)</t>
+          <t>Cotati, CA (Sonoma)</t>
         </is>
       </c>
       <c r="D57" s="49" t="inlineStr">
@@ -4322,37 +4300,37 @@
       </c>
       <c r="E57" s="50" t="inlineStr">
         <is>
+          <t>(707) 242-6922</t>
+        </is>
+      </c>
+      <c r="F57" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G57" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F57" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G57" s="49" t="inlineStr">
+      <c r="H57" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H57" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I57" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J57" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://gdlserves.com/</t>
         </is>
       </c>
       <c r="K57" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>customercare@gdlserves.com</t>
         </is>
       </c>
       <c r="L57" s="49" t="inlineStr">
@@ -4362,7 +4340,7 @@
       </c>
       <c r="M57" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Appears in Hayward cleaning-service directories. Verify legal name, phone, and commercial vs residential mix on the call.</t>
+          <t>Business line: ask for the current owner. North Bay commercial-only janitorial, carpet, floor waxing, windows, and post-construction. 321 Blodgett St, Ste A.</t>
         </is>
       </c>
       <c r="N57" s="49" t="inlineStr">
@@ -4379,7 +4357,7 @@
     <row r="58" ht="48" customHeight="1" s="47">
       <c r="A58" s="49" t="inlineStr">
         <is>
-          <t>Resourceful Janitorial and Business Solutions</t>
+          <t>Nico Janitorial</t>
         </is>
       </c>
       <c r="B58" s="49" t="inlineStr">
@@ -4389,7 +4367,7 @@
       </c>
       <c r="C58" s="49" t="inlineStr">
         <is>
-          <t>Hayward, CA (Alameda)</t>
+          <t>San Leandro, CA (Alameda)</t>
         </is>
       </c>
       <c r="D58" s="49" t="inlineStr">
@@ -4399,37 +4377,37 @@
       </c>
       <c r="E58" s="50" t="inlineStr">
         <is>
+          <t>(510) 844-4638</t>
+        </is>
+      </c>
+      <c r="F58" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G58" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="F58" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G58" s="49" t="inlineStr">
+      <c r="H58" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H58" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I58" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J58" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://www.nicojanitorial.com/</t>
         </is>
       </c>
       <c r="K58" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@nicojanitorial.com</t>
         </is>
       </c>
       <c r="L58" s="49" t="inlineStr">
@@ -4439,7 +4417,7 @@
       </c>
       <c r="M58" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Listed among Hayward commercial cleaning providers. Verify phone, website, and current operating status on the call.</t>
+          <t>Business line: ask for the current owner. East Bay commercial janitorial for offices, healthcare, schools, manufacturing, and hospitality. 933 MacArthur Blvd, Ste 1B. CA DIR JS-LR-1001308309.</t>
         </is>
       </c>
       <c r="N58" s="49" t="inlineStr">
@@ -4456,7 +4434,7 @@
     <row r="59" ht="48" customHeight="1" s="47">
       <c r="A59" s="49" t="inlineStr">
         <is>
-          <t>Peninsula Mobile Service</t>
+          <t>JLP Building Maintenance, LLC</t>
         </is>
       </c>
       <c r="B59" s="49" t="inlineStr">
@@ -4466,47 +4444,45 @@
       </c>
       <c r="C59" s="49" t="inlineStr">
         <is>
-          <t>San Mateo County, CA</t>
+          <t>Fremont, CA (Alameda)</t>
         </is>
       </c>
       <c r="D59" s="49" t="inlineStr">
         <is>
+          <t>Jorge (first name in client testimonials; surname not independently verified)</t>
+        </is>
+      </c>
+      <c r="E59" s="50" t="inlineStr">
+        <is>
+          <t>(510) 656-8300</t>
+        </is>
+      </c>
+      <c r="F59" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G59" s="49" t="n">
+        <v>20</v>
+      </c>
+      <c r="H59" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E59" s="50" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="F59" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G59" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H59" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I59" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J59" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>http://www.jlpbuilding.com/</t>
         </is>
       </c>
       <c r="K59" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@jlpbuilding.com</t>
         </is>
       </c>
       <c r="L59" s="49" t="inlineStr">
@@ -4516,7 +4492,7 @@
       </c>
       <c r="M59" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Blue Book-adjacent Peninsula building-maintenance listing. Verify commercial janitorial fit, phone, and city on the call.</t>
+          <t>Business line: ask for Jorge and confirm current ownership. East Bay/South Bay janitorial, windows, carpet, and clean-room/ESD floor care. 48834 Kato Rd, Ste 109A. Distinct from Fremont Janitorial on the prior list.</t>
         </is>
       </c>
       <c r="N59" s="49" t="inlineStr">
@@ -4533,7 +4509,7 @@
     <row r="60" ht="48" customHeight="1" s="47">
       <c r="A60" s="49" t="inlineStr">
         <is>
-          <t>Maintenance Professionals, Inc.</t>
+          <t>Extreme Janitors</t>
         </is>
       </c>
       <c r="B60" s="49" t="inlineStr">
@@ -4543,49 +4519,45 @@
       </c>
       <c r="C60" s="49" t="inlineStr">
         <is>
-          <t>San Jose / South Bay, CA</t>
+          <t>Oakland, CA (Alameda)</t>
         </is>
       </c>
       <c r="D60" s="49" t="inlineStr">
         <is>
+          <t>Abel Casanga (Founder)</t>
+        </is>
+      </c>
+      <c r="E60" s="50" t="inlineStr">
+        <is>
+          <t>(510) 842-8949</t>
+        </is>
+      </c>
+      <c r="F60" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G60" s="49" t="n">
+        <v>11</v>
+      </c>
+      <c r="H60" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="I60" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J60" s="49" t="inlineStr">
+        <is>
+          <t>https://extremejanitors.com/</t>
+        </is>
+      </c>
+      <c r="K60" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E60" s="50" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="F60" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G60" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H60" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I60" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J60" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K60" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L60" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -4593,7 +4565,7 @@
       </c>
       <c r="M60" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Blue Book-adjacent South Bay janitorial/building-maintenance listing. Verify phone, website, and ownership on the call.</t>
+          <t>Business line: ask for Abel Casanga and confirm current ownership. Oakland family-owned commercial janitorial since 2015. 2872 E 7th St.</t>
         </is>
       </c>
       <c r="N60" s="49" t="inlineStr">
@@ -4610,7 +4582,7 @@
     <row r="61" ht="48" customHeight="1" s="47">
       <c r="A61" s="49" t="inlineStr">
         <is>
-          <t>Lua's Construction &amp; Facilities</t>
+          <t>KD Janitorial Services, Inc.</t>
         </is>
       </c>
       <c r="B61" s="49" t="inlineStr">
@@ -4620,17 +4592,17 @@
       </c>
       <c r="C61" s="49" t="inlineStr">
         <is>
-          <t>San Jose, CA (Santa Clara)</t>
+          <t>Oakland, CA (Alameda); also serves SF and San Jose</t>
         </is>
       </c>
       <c r="D61" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>Kelvin Diaz (Founder/CEO)</t>
         </is>
       </c>
       <c r="E61" s="50" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>(510) 422-3260</t>
         </is>
       </c>
       <c r="F61" s="49" t="inlineStr">
@@ -4638,29 +4610,25 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G61" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="H61" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
+      <c r="G61" s="49" t="n">
+        <v>9</v>
+      </c>
+      <c r="H61" s="49" t="n">
+        <v>10</v>
       </c>
       <c r="I61" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J61" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>https://kdjanitorial.com/</t>
         </is>
       </c>
       <c r="K61" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@kdjanitorial.com</t>
         </is>
       </c>
       <c r="L61" s="49" t="inlineStr">
@@ -4670,7 +4638,7 @@
       </c>
       <c r="M61" s="49" t="inlineStr">
         <is>
-          <t>Ask for the current owner. Blue Book listing for janitorial and parking-lot maintenance. Verify phone, commercial mix, and current operating status on the call.</t>
+          <t>Business line: ask for Kelvin Diaz and confirm current ownership. Family-owned commercial/industrial cleaning since 2017. LinkedIn HQ Oakland; some materials also list Tracy (outside the nine counties).</t>
         </is>
       </c>
       <c r="N61" s="49" t="inlineStr">
@@ -4839,7 +4807,7 @@
     <row r="64" ht="48" customHeight="1" s="47">
       <c r="A64" s="49" t="inlineStr">
         <is>
-          <t>Sta-Clean</t>
+          <t>Sta-Clean Services, Inc.</t>
         </is>
       </c>
       <c r="B64" s="49" t="inlineStr">
@@ -4854,7 +4822,7 @@
       </c>
       <c r="D64" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>Brant (owner first name published; surname not independently verified)</t>
         </is>
       </c>
       <c r="E64" s="50" t="inlineStr">
@@ -4897,7 +4865,7 @@
       </c>
       <c r="M64" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Commercial/office janitorial since 1981 for SF, Marin, Sonoma, and Contra Costa offices, schools, health clubs, and warehouses.</t>
+          <t>Business line: ask for Brant and confirm current ownership. Commercial/office janitorial since 1981 for SF, Marin, Sonoma, and Contra Costa.</t>
         </is>
       </c>
       <c r="N64" s="49" t="inlineStr">
@@ -4914,7 +4882,7 @@
     <row r="65" ht="48" customHeight="1" s="47">
       <c r="A65" s="49" t="inlineStr">
         <is>
-          <t>Consolidated Cleaning Solutions Inc.</t>
+          <t>Consolidated Cleaning Solutions, Inc.</t>
         </is>
       </c>
       <c r="B65" s="49" t="inlineStr">
@@ -4929,44 +4897,42 @@
       </c>
       <c r="D65" s="49" t="inlineStr">
         <is>
+          <t>Martin Gonzalez</t>
+        </is>
+      </c>
+      <c r="E65" s="50" t="inlineStr">
+        <is>
+          <t>(510) 969-7416</t>
+        </is>
+      </c>
+      <c r="F65" s="49" t="inlineStr">
+        <is>
+          <t>Business Line</t>
+        </is>
+      </c>
+      <c r="G65" s="49" t="n">
+        <v>42</v>
+      </c>
+      <c r="H65" s="49" t="inlineStr">
+        <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="E65" s="50" t="inlineStr">
-        <is>
-          <t>(510) 969-7416</t>
-        </is>
-      </c>
-      <c r="F65" s="49" t="inlineStr">
-        <is>
-          <t>Business Line</t>
-        </is>
-      </c>
-      <c r="G65" s="49" t="inlineStr">
+      <c r="I65" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J65" s="49" t="inlineStr">
+        <is>
+          <t>https://consolidated-cleaning.com/</t>
+        </is>
+      </c>
+      <c r="K65" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H65" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="I65" s="49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J65" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
-      <c r="K65" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="L65" s="49" t="inlineStr">
         <is>
           <t>New</t>
@@ -4974,7 +4940,7 @@
       </c>
       <c r="M65" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Public listings place the firm at 406 Pendleton Way, Oakland. Verify website, legal status, and commercial janitorial mix on the call.</t>
+          <t>Business line: ask for Martin Gonzalez and confirm current ownership. Minority-owned commercial janitorial since 1984; windows, carpet, pressure washing, and construction cleaning.</t>
         </is>
       </c>
       <c r="N65" s="49" t="inlineStr">
@@ -4991,7 +4957,7 @@
     <row r="66" ht="48" customHeight="1" s="47">
       <c r="A66" s="49" t="inlineStr">
         <is>
-          <t>American Empire Building Services</t>
+          <t>Global Maintenance Resources</t>
         </is>
       </c>
       <c r="B66" s="49" t="inlineStr">
@@ -5001,7 +4967,7 @@
       </c>
       <c r="C66" s="49" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Union City, CA (Alameda)</t>
         </is>
       </c>
       <c r="D66" s="49" t="inlineStr">
@@ -5011,7 +4977,7 @@
       </c>
       <c r="E66" s="50" t="inlineStr">
         <is>
-          <t>(415) 536-7842</t>
+          <t>(510) 377-6085</t>
         </is>
       </c>
       <c r="F66" s="49" t="inlineStr">
@@ -5019,29 +4985,27 @@
           <t>Business Line</t>
         </is>
       </c>
-      <c r="G66" s="49" t="inlineStr">
+      <c r="G66" s="49" t="n">
+        <v>25</v>
+      </c>
+      <c r="H66" s="49" t="inlineStr">
         <is>
           <t>Not publicly verified</t>
         </is>
       </c>
-      <c r="H66" s="49" t="inlineStr">
-        <is>
-          <t>Not publicly verified</t>
-        </is>
-      </c>
       <c r="I66" s="49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J66" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>http://gmresources.com/</t>
         </is>
       </c>
       <c r="K66" s="49" t="inlineStr">
         <is>
-          <t>Not publicly verified</t>
+          <t>info@GMResources.com</t>
         </is>
       </c>
       <c r="L66" s="49" t="inlineStr">
@@ -5051,7 +5015,7 @@
       </c>
       <c r="M66" s="49" t="inlineStr">
         <is>
-          <t>Business line: ask for the current owner. Public listings place the firm at 440 Bryant St, San Francisco. Verify website and current operating status on the call.</t>
+          <t>Business line: ask for the current owner. Commercial janitorial and building maintenance since 2001. 1684 Decoto Rd #314. Offices, community centers, fitness, and HOA common areas.</t>
         </is>
       </c>
       <c r="N66" s="49" t="inlineStr">

</xml_diff>